<commit_message>
add leaf scans and labels
</commit_message>
<xml_diff>
--- a/hoagland_recipes/NxPxI_hoagland_highN.xlsx
+++ b/hoagland_recipes/NxPxI_hoagland_highN.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eaperkowski/git/2026_NxPxI/hoagland_recipes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{922BCC09-28C3-2240-A8FD-55FEDBEC06BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7E74273-93D2-B445-9A65-2CA28DB437BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1480" yWindow="660" windowWidth="28500" windowHeight="18980" activeTab="6" xr2:uid="{EA5B7CD4-0592-B14D-A568-E53194DF6487}"/>
+    <workbookView xWindow="34280" yWindow="5200" windowWidth="28500" windowHeight="18980" activeTab="6" xr2:uid="{EA5B7CD4-0592-B14D-A568-E53194DF6487}"/>
   </bookViews>
   <sheets>
     <sheet name="Stock solutions" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
     <sheet name="210 ppm N, 62 ppm P" sheetId="8" r:id="rId6"/>
     <sheet name="210 ppm N, 93 ppm P" sheetId="9" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="62">
   <si>
     <t>compound name and stock solution  molarity</t>
   </si>
@@ -1169,6 +1169,9 @@
   </si>
   <si>
     <t>macro</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -1368,28 +1371,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1909,7 +1891,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F7E91A3-BC3E-BA4A-95DE-642736502BE5}">
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30.6640625" bestFit="1" customWidth="1"/>
@@ -1917,13 +1899,13 @@
     <col min="3" max="3" width="8.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="8" t="s">
         <v>18</v>
       </c>
       <c r="B1" s="8"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -1940,7 +1922,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -1956,8 +1938,12 @@
       <c r="E3" s="9">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F3">
+        <f>D3*20</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -1971,11 +1957,15 @@
         <v>2</v>
       </c>
       <c r="E4" s="9">
-        <f t="shared" ref="E3:E5" si="0">(C4*1000)/(1000/(B4*D4))</f>
+        <f t="shared" ref="E4:E5" si="0">(C4*1000)/(1000/(B4*D4))</f>
         <v>404.4</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F4">
+        <f t="shared" ref="F4:F15" si="1">D4*20</f>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>26</v>
       </c>
@@ -1992,8 +1982,12 @@
         <f t="shared" si="0"/>
         <v>656.35199999999998</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F5">
+        <f t="shared" si="1"/>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -2010,13 +2004,27 @@
         <f>(C6*1000)/(1000/(B6*D6))</f>
         <v>120.06450000000001</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F6">
+        <f t="shared" si="1"/>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F7">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F8">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -2032,8 +2040,12 @@
       <c r="E9" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F9" t="e">
+        <f t="shared" si="1"/>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>29</v>
       </c>
@@ -2049,8 +2061,12 @@
       <c r="E10" s="9">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>30</v>
       </c>
@@ -2066,8 +2082,12 @@
       <c r="E11" s="9">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>31</v>
       </c>
@@ -2083,8 +2103,12 @@
       <c r="E12" s="9">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>32</v>
       </c>
@@ -2098,11 +2122,15 @@
         <v>1</v>
       </c>
       <c r="E13" s="9">
-        <f t="shared" ref="E12:E15" si="1">(C13*1000)/(1000/(B13*D13))</f>
+        <f t="shared" ref="E13:E15" si="2">(C13*1000)/(1000/(B13*D13))</f>
         <v>492.96</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F13">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>33</v>
       </c>
@@ -2113,8 +2141,12 @@
         <v>1</v>
       </c>
       <c r="E14" s="9"/>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F14">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>34</v>
       </c>
@@ -2125,8 +2157,12 @@
         <v>1</v>
       </c>
       <c r="E15" s="9">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <f t="shared" si="1"/>
+        <v>20</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
@@ -2202,7 +2238,7 @@
         <v>2</v>
       </c>
       <c r="E21" s="9">
-        <f t="shared" ref="E19:E27" si="2">(C21*1000)/(1000/(B21*D21))</f>
+        <f t="shared" ref="E21:E25" si="3">(C21*1000)/(1000/(B21*D21))</f>
         <v>156.37719999999999</v>
       </c>
     </row>
@@ -2221,7 +2257,7 @@
         <v>2</v>
       </c>
       <c r="E22" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>56.024000000000001</v>
       </c>
     </row>
@@ -2240,7 +2276,7 @@
         <v>2</v>
       </c>
       <c r="E23" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>160.31200000000001</v>
       </c>
     </row>
@@ -2259,7 +2295,7 @@
         <v>2</v>
       </c>
       <c r="E24" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>112.048</v>
       </c>
     </row>
@@ -2278,7 +2314,7 @@
         <v>1.5</v>
       </c>
       <c r="E25" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>42.018000000000001</v>
       </c>
     </row>
@@ -2387,7 +2423,7 @@
         <v>1</v>
       </c>
       <c r="E31" s="9">
-        <f t="shared" ref="E26:E32" si="3">(C31*1000)/(1000/(B31*D31))</f>
+        <f t="shared" ref="E31:E32" si="4">(C31*1000)/(1000/(B31*D31))</f>
         <v>48.61</v>
       </c>
     </row>
@@ -2406,7 +2442,7 @@
         <v>1</v>
       </c>
       <c r="E32" s="9">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>64.13</v>
       </c>
     </row>
@@ -2533,19 +2569,19 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{516136DE-12C0-BC4C-B963-A9701A317B59}">
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="8" t="s">
         <v>18</v>
       </c>
       <c r="B1" s="8"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -2562,7 +2598,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -2578,8 +2614,12 @@
       <c r="E3" s="9">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F3">
+        <f>D3*20</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -2593,11 +2633,15 @@
         <v>2</v>
       </c>
       <c r="E4" s="9">
-        <f t="shared" ref="E3:E5" si="0">(C4*1000)/(1000/(B4*D4))</f>
+        <f t="shared" ref="E4:E5" si="0">(C4*1000)/(1000/(B4*D4))</f>
         <v>404.4</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F4">
+        <f t="shared" ref="F4:F15" si="1">D4*20</f>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>26</v>
       </c>
@@ -2614,8 +2658,12 @@
         <f t="shared" si="0"/>
         <v>656.35199999999998</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F5">
+        <f t="shared" si="1"/>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -2632,13 +2680,27 @@
         <f>(C6*1000)/(1000/(B6*D6))</f>
         <v>110.45933999999998</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F6">
+        <f t="shared" si="1"/>
+        <v>27.599999999999998</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F7">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F8">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -2654,8 +2716,12 @@
       <c r="E9" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F9" t="e">
+        <f t="shared" si="1"/>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>29</v>
       </c>
@@ -2671,8 +2737,12 @@
       <c r="E10" s="9">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>30</v>
       </c>
@@ -2688,8 +2758,12 @@
       <c r="E11" s="9">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>31</v>
       </c>
@@ -2705,8 +2779,12 @@
       <c r="E12" s="9">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>32</v>
       </c>
@@ -2720,11 +2798,15 @@
         <v>1</v>
       </c>
       <c r="E13" s="9">
-        <f t="shared" ref="E12:E15" si="1">(C13*1000)/(1000/(B13*D13))</f>
+        <f t="shared" ref="E13:E15" si="2">(C13*1000)/(1000/(B13*D13))</f>
         <v>492.96</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F13">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>33</v>
       </c>
@@ -2735,8 +2817,12 @@
         <v>1</v>
       </c>
       <c r="E14" s="9"/>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F14">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>34</v>
       </c>
@@ -2747,8 +2833,12 @@
         <v>1</v>
       </c>
       <c r="E15" s="9">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <f t="shared" si="1"/>
+        <v>20</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
@@ -2788,7 +2878,7 @@
         <v>0.25</v>
       </c>
       <c r="E19" s="9">
-        <f t="shared" ref="E19:E25" si="2">(C19*1000)/(1000/(B19*D19))</f>
+        <f t="shared" ref="E19:E25" si="3">(C19*1000)/(1000/(B19*D19))</f>
         <v>3.5015000000000001</v>
       </c>
     </row>
@@ -2807,7 +2897,7 @@
         <v>0.25</v>
       </c>
       <c r="E20" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>7.7434250000000002</v>
       </c>
     </row>
@@ -2826,7 +2916,7 @@
         <v>2</v>
       </c>
       <c r="E21" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>156.37719999999999</v>
       </c>
     </row>
@@ -2845,7 +2935,7 @@
         <v>2</v>
       </c>
       <c r="E22" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>56.024000000000001</v>
       </c>
     </row>
@@ -2864,7 +2954,7 @@
         <v>2</v>
       </c>
       <c r="E23" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>160.31200000000001</v>
       </c>
     </row>
@@ -2883,7 +2973,7 @@
         <v>2</v>
       </c>
       <c r="E24" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>112.048</v>
       </c>
     </row>
@@ -2902,7 +2992,7 @@
         <v>1.38</v>
       </c>
       <c r="E25" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>38.656559999999999</v>
       </c>
     </row>
@@ -3011,7 +3101,7 @@
         <v>1</v>
       </c>
       <c r="E31" s="9">
-        <f t="shared" ref="E26:E32" si="3">(C31*1000)/(1000/(B31*D31))</f>
+        <f t="shared" ref="E31:E32" si="4">(C31*1000)/(1000/(B31*D31))</f>
         <v>48.61</v>
       </c>
     </row>
@@ -3030,7 +3120,7 @@
         <v>1</v>
       </c>
       <c r="E32" s="9">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>64.13</v>
       </c>
     </row>
@@ -3158,19 +3248,19 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC620572-E7E9-C149-A071-72B5F47728B3}">
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="8" t="s">
         <v>18</v>
       </c>
       <c r="B1" s="8"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -3187,7 +3277,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -3204,8 +3294,12 @@
         <f t="shared" ref="E3:E5" si="0">(C3*1000)/(1000/(B3*D3))</f>
         <v>57.65</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F3">
+        <f>D3*20</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -3222,8 +3316,12 @@
         <f t="shared" si="0"/>
         <v>404.4</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F4">
+        <f t="shared" ref="F4:F15" si="1">D4*20</f>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>26</v>
       </c>
@@ -3240,8 +3338,12 @@
         <f t="shared" si="0"/>
         <v>656.35199999999998</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F5">
+        <f t="shared" si="1"/>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -3258,13 +3360,27 @@
         <f>(C6*1000)/(1000/(B6*D6))</f>
         <v>100.05374999999999</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F6">
+        <f t="shared" si="1"/>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F7">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F8">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -3280,8 +3396,12 @@
       <c r="E9" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F9" t="e">
+        <f t="shared" si="1"/>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>29</v>
       </c>
@@ -3297,8 +3417,12 @@
       <c r="E10" s="9">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>30</v>
       </c>
@@ -3314,8 +3438,12 @@
       <c r="E11" s="9">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>31</v>
       </c>
@@ -3331,8 +3459,12 @@
       <c r="E12" s="9">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>32</v>
       </c>
@@ -3346,11 +3478,15 @@
         <v>1</v>
       </c>
       <c r="E13" s="9">
-        <f t="shared" ref="E12:E15" si="1">(C13*1000)/(1000/(B13*D13))</f>
+        <f t="shared" ref="E13:E15" si="2">(C13*1000)/(1000/(B13*D13))</f>
         <v>492.96</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F13">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>33</v>
       </c>
@@ -3361,8 +3497,12 @@
         <v>1</v>
       </c>
       <c r="E14" s="9"/>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F14">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>34</v>
       </c>
@@ -3373,8 +3513,12 @@
         <v>1</v>
       </c>
       <c r="E15" s="9">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <f t="shared" si="1"/>
+        <v>20</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
@@ -3414,7 +3558,7 @@
         <v>0.5</v>
       </c>
       <c r="E19" s="9">
-        <f t="shared" ref="E19:E30" si="2">(C19*1000)/(1000/(B19*D19))</f>
+        <f t="shared" ref="E19:E25" si="3">(C19*1000)/(1000/(B19*D19))</f>
         <v>7.0030000000000001</v>
       </c>
     </row>
@@ -3433,7 +3577,7 @@
         <v>0.5</v>
       </c>
       <c r="E20" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>15.48685</v>
       </c>
     </row>
@@ -3452,7 +3596,7 @@
         <v>2</v>
       </c>
       <c r="E21" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>156.37719999999999</v>
       </c>
     </row>
@@ -3471,7 +3615,7 @@
         <v>2</v>
       </c>
       <c r="E22" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>56.024000000000001</v>
       </c>
     </row>
@@ -3490,7 +3634,7 @@
         <v>2</v>
       </c>
       <c r="E23" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>160.31200000000001</v>
       </c>
     </row>
@@ -3509,7 +3653,7 @@
         <v>2</v>
       </c>
       <c r="E24" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>112.048</v>
       </c>
     </row>
@@ -3528,7 +3672,7 @@
         <v>1.25</v>
       </c>
       <c r="E25" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>35.015000000000001</v>
       </c>
     </row>
@@ -3637,7 +3781,7 @@
         <v>1</v>
       </c>
       <c r="E31" s="9">
-        <f t="shared" ref="E26:E32" si="3">(C31*1000)/(1000/(B31*D31))</f>
+        <f t="shared" ref="E31:E32" si="4">(C31*1000)/(1000/(B31*D31))</f>
         <v>48.61</v>
       </c>
     </row>
@@ -3656,7 +3800,7 @@
         <v>1</v>
       </c>
       <c r="E32" s="9">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>64.13</v>
       </c>
     </row>
@@ -3784,19 +3928,19 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C097AD85-1C36-514C-8973-F08DE1511404}">
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="8" t="s">
         <v>18</v>
       </c>
       <c r="B1" s="8"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -3813,7 +3957,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -3830,8 +3974,12 @@
         <f>(C3*1000)/(1000/(B3*D3))</f>
         <v>115.3</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F3">
+        <f>D3*20</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -3845,11 +3993,15 @@
         <v>2</v>
       </c>
       <c r="E4" s="9">
-        <f t="shared" ref="E3:E5" si="0">(C4*1000)/(1000/(B4*D4))</f>
+        <f t="shared" ref="E4:E5" si="0">(C4*1000)/(1000/(B4*D4))</f>
         <v>404.4</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F4">
+        <f t="shared" ref="F4:F20" si="1">D4*20</f>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>26</v>
       </c>
@@ -3866,8 +4018,12 @@
         <f t="shared" si="0"/>
         <v>656.35199999999998</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F5">
+        <f t="shared" si="1"/>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -3884,13 +4040,27 @@
         <f>(C6*1000)/(1000/(B6*D6))</f>
         <v>80.043000000000006</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F6">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F7">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F8">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -3906,8 +4076,12 @@
       <c r="E9" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F9" t="e">
+        <f t="shared" si="1"/>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>29</v>
       </c>
@@ -3923,8 +4097,12 @@
       <c r="E10" s="9">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>30</v>
       </c>
@@ -3940,8 +4118,12 @@
       <c r="E11" s="9">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>31</v>
       </c>
@@ -3957,8 +4139,12 @@
       <c r="E12" s="9">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>32</v>
       </c>
@@ -3972,11 +4158,15 @@
         <v>1</v>
       </c>
       <c r="E13" s="9">
-        <f t="shared" ref="E13:E16" si="1">(C13*1000)/(1000/(B13*D13))</f>
+        <f t="shared" ref="E13:E15" si="2">(C13*1000)/(1000/(B13*D13))</f>
         <v>492.96</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F13">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>33</v>
       </c>
@@ -3987,8 +4177,12 @@
         <v>1</v>
       </c>
       <c r="E14" s="9"/>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F14">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>34</v>
       </c>
@@ -3999,16 +4193,30 @@
         <v>1</v>
       </c>
       <c r="E15" s="9">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F16">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="8" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>36</v>
       </c>
@@ -4024,8 +4232,12 @@
       <c r="E18" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F18" t="e">
+        <f t="shared" si="1"/>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -4043,8 +4255,12 @@
         <f>(C19*1000)/(1000/(B19*D19))</f>
         <v>14.006</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F19">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>38</v>
       </c>
@@ -4059,11 +4275,15 @@
         <v>1</v>
       </c>
       <c r="E20" s="9">
-        <f t="shared" ref="E19:E30" si="2">(C20*1000)/(1000/(B20*D20))</f>
+        <f t="shared" ref="E20:E25" si="3">(C20*1000)/(1000/(B20*D20))</f>
         <v>30.973700000000001</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F20">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>39</v>
       </c>
@@ -4078,11 +4298,11 @@
         <v>2</v>
       </c>
       <c r="E21" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>156.37719999999999</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>40</v>
       </c>
@@ -4097,11 +4317,11 @@
         <v>2</v>
       </c>
       <c r="E22" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>56.024000000000001</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>41</v>
       </c>
@@ -4116,11 +4336,11 @@
         <v>2</v>
       </c>
       <c r="E23" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>160.31200000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>42</v>
       </c>
@@ -4135,11 +4355,11 @@
         <v>2</v>
       </c>
       <c r="E24" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>112.048</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>43</v>
       </c>
@@ -4154,11 +4374,11 @@
         <v>1</v>
       </c>
       <c r="E25" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>28.012</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>44</v>
       </c>
@@ -4176,7 +4396,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>45</v>
       </c>
@@ -4194,7 +4414,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>46</v>
       </c>
@@ -4212,7 +4432,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>47</v>
       </c>
@@ -4230,7 +4450,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>48</v>
       </c>
@@ -4248,7 +4468,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>49</v>
       </c>
@@ -4263,11 +4483,11 @@
         <v>1</v>
       </c>
       <c r="E31" s="9">
-        <f t="shared" ref="E31:E37" si="3">(C31*1000)/(1000/(B31*D31))</f>
+        <f t="shared" ref="E31:E32" si="4">(C31*1000)/(1000/(B31*D31))</f>
         <v>48.61</v>
       </c>
     </row>
-    <row r="32" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>50</v>
       </c>
@@ -4282,7 +4502,7 @@
         <v>1</v>
       </c>
       <c r="E32" s="9">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>64.13</v>
       </c>
     </row>
@@ -4410,19 +4630,19 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74D762CA-CBA6-4F4B-B6C7-FFC0A474BA45}">
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="8" t="s">
         <v>18</v>
       </c>
       <c r="B1" s="8"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -4439,7 +4659,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -4456,8 +4676,12 @@
         <f>(C3*1000)/(1000/(B3*D3))</f>
         <v>230.6</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F3">
+        <f>D3*2</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -4474,8 +4698,12 @@
         <f t="shared" ref="E4:E5" si="0">(C4*1000)/(1000/(B4*D4))</f>
         <v>404.4</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F4">
+        <f t="shared" ref="F4:F15" si="1">D4*2</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>26</v>
       </c>
@@ -4492,8 +4720,12 @@
         <f t="shared" si="0"/>
         <v>656.35199999999998</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F5">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -4510,13 +4742,27 @@
         <f>(C6*1000)/(1000/(B6*D6))</f>
         <v>40.021500000000003</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F6">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F7">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F8">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -4532,8 +4778,12 @@
       <c r="E9" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F9" t="e">
+        <f t="shared" si="1"/>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>29</v>
       </c>
@@ -4549,8 +4799,12 @@
       <c r="E10" s="9">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>30</v>
       </c>
@@ -4566,8 +4820,12 @@
       <c r="E11" s="9">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>31</v>
       </c>
@@ -4583,8 +4841,12 @@
       <c r="E12" s="9">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>32</v>
       </c>
@@ -4598,11 +4860,15 @@
         <v>1</v>
       </c>
       <c r="E13" s="9">
-        <f t="shared" ref="E13:E16" si="1">(C13*1000)/(1000/(B13*D13))</f>
+        <f t="shared" ref="E13:E15" si="2">(C13*1000)/(1000/(B13*D13))</f>
         <v>492.96</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F13">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>33</v>
       </c>
@@ -4613,8 +4879,12 @@
         <v>1</v>
       </c>
       <c r="E14" s="9"/>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F14">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>34</v>
       </c>
@@ -4625,8 +4895,12 @@
         <v>1</v>
       </c>
       <c r="E15" s="9">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <f t="shared" si="1"/>
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
@@ -4685,7 +4959,7 @@
         <v>2</v>
       </c>
       <c r="E20" s="9">
-        <f t="shared" ref="E20:E31" si="2">(C20*1000)/(1000/(B20*D20))</f>
+        <f t="shared" ref="E20:E25" si="3">(C20*1000)/(1000/(B20*D20))</f>
         <v>61.947400000000002</v>
       </c>
     </row>
@@ -4704,7 +4978,7 @@
         <v>2</v>
       </c>
       <c r="E21" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>156.37719999999999</v>
       </c>
     </row>
@@ -4723,7 +4997,7 @@
         <v>2</v>
       </c>
       <c r="E22" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>56.024000000000001</v>
       </c>
     </row>
@@ -4742,7 +5016,7 @@
         <v>2</v>
       </c>
       <c r="E23" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>160.31200000000001</v>
       </c>
     </row>
@@ -4761,7 +5035,7 @@
         <v>2</v>
       </c>
       <c r="E24" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>112.048</v>
       </c>
     </row>
@@ -4780,7 +5054,7 @@
         <v>0.5</v>
       </c>
       <c r="E25" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>14.006</v>
       </c>
     </row>
@@ -4889,7 +5163,7 @@
         <v>1</v>
       </c>
       <c r="E31" s="9">
-        <f t="shared" ref="E31:E37" si="3">(C31*1000)/(1000/(B31*D31))</f>
+        <f t="shared" ref="E31:E32" si="4">(C31*1000)/(1000/(B31*D31))</f>
         <v>48.61</v>
       </c>
     </row>
@@ -4908,7 +5182,7 @@
         <v>1</v>
       </c>
       <c r="E32" s="9">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>64.13</v>
       </c>
     </row>
@@ -5036,19 +5310,19 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF539455-23E4-0843-B935-AE858235A388}">
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="8" t="s">
         <v>18</v>
       </c>
       <c r="B1" s="8"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -5065,7 +5339,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -5082,8 +5356,11 @@
         <f>(C3*1000)/(1000/(B3*D3))</f>
         <v>345.90000000000003</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -5100,8 +5377,12 @@
         <f t="shared" ref="E4:E5" si="0">(C4*1000)/(1000/(B4*D4))</f>
         <v>404.4</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F4">
+        <f t="shared" ref="F4:F15" si="1">D4*2</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>26</v>
       </c>
@@ -5118,8 +5399,12 @@
         <f t="shared" si="0"/>
         <v>656.35199999999998</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F5">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -5135,13 +5420,27 @@
       <c r="E6" s="9">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F7">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F8">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -5157,8 +5456,12 @@
       <c r="E9" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F9" t="e">
+        <f t="shared" si="1"/>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>29</v>
       </c>
@@ -5174,8 +5477,12 @@
       <c r="E10" s="9">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>30</v>
       </c>
@@ -5191,8 +5498,12 @@
       <c r="E11" s="9">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>31</v>
       </c>
@@ -5208,8 +5519,12 @@
       <c r="E12" s="9">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="F12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>32</v>
       </c>
@@ -5223,11 +5538,15 @@
         <v>1</v>
       </c>
       <c r="E13" s="9">
-        <f t="shared" ref="E13:E16" si="1">(C13*1000)/(1000/(B13*D13))</f>
+        <f t="shared" ref="E13:E15" si="2">(C13*1000)/(1000/(B13*D13))</f>
         <v>492.96</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F13">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>33</v>
       </c>
@@ -5238,8 +5557,12 @@
         <v>1</v>
       </c>
       <c r="E14" s="9"/>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F14">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>34</v>
       </c>
@@ -5250,8 +5573,12 @@
         <v>1</v>
       </c>
       <c r="E15" s="9">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <f t="shared" si="1"/>
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
@@ -5310,7 +5637,7 @@
         <v>3</v>
       </c>
       <c r="E20" s="9">
-        <f t="shared" ref="E20:E31" si="2">(C20*1000)/(1000/(B20*D20))</f>
+        <f t="shared" ref="E20:E24" si="3">(C20*1000)/(1000/(B20*D20))</f>
         <v>92.92110000000001</v>
       </c>
     </row>
@@ -5329,7 +5656,7 @@
         <v>2</v>
       </c>
       <c r="E21" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>156.37719999999999</v>
       </c>
     </row>
@@ -5348,7 +5675,7 @@
         <v>2</v>
       </c>
       <c r="E22" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>56.024000000000001</v>
       </c>
     </row>
@@ -5367,7 +5694,7 @@
         <v>2</v>
       </c>
       <c r="E23" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>160.31200000000001</v>
       </c>
     </row>
@@ -5386,7 +5713,7 @@
         <v>2</v>
       </c>
       <c r="E24" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>112.048</v>
       </c>
     </row>
@@ -5513,7 +5840,7 @@
         <v>1</v>
       </c>
       <c r="E31" s="9">
-        <f t="shared" ref="E31:E37" si="3">(C31*1000)/(1000/(B31*D31))</f>
+        <f t="shared" ref="E31:E32" si="4">(C31*1000)/(1000/(B31*D31))</f>
         <v>48.61</v>
       </c>
     </row>
@@ -5532,7 +5859,7 @@
         <v>1</v>
       </c>
       <c r="E32" s="9">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>64.13</v>
       </c>
     </row>

</xml_diff>